<commit_message>
feat: extrai ID pedido Shopee/TikTok da planilha (280 ordens), corrige canais de venda
</commit_message>
<xml_diff>
--- a/data/excel/Backup_Dados_Completos.xlsx
+++ b/data/excel/Backup_Dados_Completos.xlsx
@@ -29005,7 +29005,7 @@
         <v>18.5</v>
       </c>
       <c r="H3" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I3" t="str">
         <v>money</v>
@@ -30368,7 +30368,7 @@
         <v>3.1</v>
       </c>
       <c r="H50" t="str">
-        <v>Shopee CPF</v>
+        <v/>
       </c>
       <c r="I50" t="str">
         <v>money</v>
@@ -30397,7 +30397,7 @@
         <v>28.3</v>
       </c>
       <c r="H51" t="str">
-        <v>Shopee CPF</v>
+        <v/>
       </c>
       <c r="I51" t="str">
         <v>money</v>
@@ -30426,7 +30426,7 @@
         <v>3.1</v>
       </c>
       <c r="H52" t="str">
-        <v>Shopee CPF</v>
+        <v/>
       </c>
       <c r="I52" t="str">
         <v>money</v>
@@ -30455,7 +30455,7 @@
         <v>3.1</v>
       </c>
       <c r="H53" t="str">
-        <v>Shopee CPF</v>
+        <v/>
       </c>
       <c r="I53" t="str">
         <v>money</v>
@@ -30484,7 +30484,7 @@
         <v>9.39</v>
       </c>
       <c r="H54" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I54" t="str">
         <v>money</v>
@@ -30542,7 +30542,7 @@
         <v>3</v>
       </c>
       <c r="H56" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I56" t="str">
         <v>money</v>
@@ -31615,7 +31615,7 @@
         <v>6.7</v>
       </c>
       <c r="H93" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I93" t="str">
         <v>money</v>
@@ -31702,7 +31702,7 @@
         <v>7.41</v>
       </c>
       <c r="H96" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I96" t="str">
         <v>money</v>
@@ -38227,7 +38227,7 @@
         <v>7.72</v>
       </c>
       <c r="H321" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I321" t="str">
         <v>money</v>
@@ -38256,7 +38256,7 @@
         <v>22.35</v>
       </c>
       <c r="H322" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I322" t="str">
         <v>money</v>
@@ -38285,7 +38285,7 @@
         <v>1.89</v>
       </c>
       <c r="H323" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I323" t="str">
         <v>money</v>
@@ -38517,7 +38517,7 @@
         <v>8.22</v>
       </c>
       <c r="H331" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I331" t="str">
         <v>money</v>
@@ -38546,7 +38546,7 @@
         <v>4.71</v>
       </c>
       <c r="H332" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I332" t="str">
         <v>money</v>
@@ -38807,7 +38807,7 @@
         <v>6</v>
       </c>
       <c r="H341" t="str">
-        <v>shopee</v>
+        <v/>
       </c>
       <c r="I341" t="str">
         <v>money</v>
@@ -49914,7 +49914,7 @@
         <v>135</v>
       </c>
       <c r="H724" t="str">
-        <v>shopee</v>
+        <v/>
       </c>
       <c r="I724" t="str">
         <v>money</v>
@@ -50320,7 +50320,7 @@
         <v>72</v>
       </c>
       <c r="H738" t="str">
-        <v>shopee</v>
+        <v/>
       </c>
       <c r="I738" t="str">
         <v>money</v>
@@ -50900,7 +50900,7 @@
         <v>65</v>
       </c>
       <c r="H758" t="str">
-        <v>shopee</v>
+        <v/>
       </c>
       <c r="I758" t="str">
         <v>money</v>
@@ -51828,7 +51828,7 @@
         <v>68.38</v>
       </c>
       <c r="H790" t="str">
-        <v>shopee</v>
+        <v/>
       </c>
       <c r="I790" t="str">
         <v>money</v>
@@ -73027,7 +73027,7 @@
         <v>361.2</v>
       </c>
       <c r="H1521" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1521" t="str">
         <v>money</v>
@@ -73056,7 +73056,7 @@
         <v>61.5</v>
       </c>
       <c r="H1522" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1522" t="str">
         <v>money</v>
@@ -73085,7 +73085,7 @@
         <v>2.76</v>
       </c>
       <c r="H1523" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1523" t="str">
         <v>money</v>
@@ -73114,7 +73114,7 @@
         <v>91</v>
       </c>
       <c r="H1524" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1524" t="str">
         <v>money</v>
@@ -73143,7 +73143,7 @@
         <v>2.26</v>
       </c>
       <c r="H1525" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1525" t="str">
         <v>money</v>
@@ -73172,7 +73172,7 @@
         <v>40</v>
       </c>
       <c r="H1526" t="str">
-        <v>tiktok</v>
+        <v/>
       </c>
       <c r="I1526" t="str">
         <v>money</v>
@@ -73201,7 +73201,7 @@
         <v>84.4</v>
       </c>
       <c r="H1527" t="str">
-        <v>tiktok</v>
+        <v/>
       </c>
       <c r="I1527" t="str">
         <v>money</v>
@@ -73230,7 +73230,7 @@
         <v>97.6</v>
       </c>
       <c r="H1528" t="str">
-        <v>tiktok</v>
+        <v/>
       </c>
       <c r="I1528" t="str">
         <v>money</v>
@@ -73259,7 +73259,7 @@
         <v>54</v>
       </c>
       <c r="H1529" t="str">
-        <v>tiktok</v>
+        <v/>
       </c>
       <c r="I1529" t="str">
         <v>money</v>
@@ -73288,7 +73288,7 @@
         <v>1.19</v>
       </c>
       <c r="H1530" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1530" t="str">
         <v>money</v>
@@ -73317,7 +73317,7 @@
         <v>4.96</v>
       </c>
       <c r="H1531" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1531" t="str">
         <v>money</v>
@@ -73346,7 +73346,7 @@
         <v>15.75</v>
       </c>
       <c r="H1532" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1532" t="str">
         <v>money</v>
@@ -73375,7 +73375,7 @@
         <v>3.87</v>
       </c>
       <c r="H1533" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1533" t="str">
         <v>money</v>
@@ -73404,7 +73404,7 @@
         <v>4.96</v>
       </c>
       <c r="H1534" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1534" t="str">
         <v>money</v>
@@ -73520,7 +73520,7 @@
         <v>3.76</v>
       </c>
       <c r="H1538" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1538" t="str">
         <v>money</v>
@@ -73549,7 +73549,7 @@
         <v>8.62</v>
       </c>
       <c r="H1539" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1539" t="str">
         <v>money</v>
@@ -73578,7 +73578,7 @@
         <v>60.25</v>
       </c>
       <c r="H1540" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1540" t="str">
         <v>money</v>
@@ -73868,7 +73868,7 @@
         <v>8.37</v>
       </c>
       <c r="H1550" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1550" t="str">
         <v>money</v>
@@ -73897,7 +73897,7 @@
         <v>18.62</v>
       </c>
       <c r="H1551" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1551" t="str">
         <v>money</v>
@@ -73926,7 +73926,7 @@
         <v>18.62</v>
       </c>
       <c r="H1552" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1552" t="str">
         <v>money</v>
@@ -73955,7 +73955,7 @@
         <v>18.62</v>
       </c>
       <c r="H1553" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1553" t="str">
         <v>money</v>
@@ -73984,7 +73984,7 @@
         <v>18.62</v>
       </c>
       <c r="H1554" t="str">
-        <v>Shopee</v>
+        <v/>
       </c>
       <c r="I1554" t="str">
         <v>money</v>
@@ -74013,7 +74013,7 @@
         <v>23.2</v>
       </c>
       <c r="H1555" t="str">
-        <v>tiktok</v>
+        <v/>
       </c>
       <c r="I1555" t="str">
         <v>money</v>
@@ -74216,7 +74216,7 @@
         <v>28.62</v>
       </c>
       <c r="H1562" t="str">
-        <v>251024UFEQ5C37</v>
+        <v/>
       </c>
       <c r="I1562" t="str">
         <v>money</v>
@@ -74245,7 +74245,7 @@
         <v>28.62</v>
       </c>
       <c r="H1563" t="str">
-        <v>251023SA4CE2K2</v>
+        <v/>
       </c>
       <c r="I1563" t="str">
         <v>money</v>
@@ -74274,7 +74274,7 @@
         <v>28.62</v>
       </c>
       <c r="H1564" t="str">
-        <v>251023S43AH3PT</v>
+        <v/>
       </c>
       <c r="I1564" t="str">
         <v>money</v>
@@ -74303,7 +74303,7 @@
         <v>28.62</v>
       </c>
       <c r="H1565" t="str">
-        <v>2510250T39QW0M</v>
+        <v/>
       </c>
       <c r="I1565" t="str">
         <v>money</v>
@@ -74332,7 +74332,7 @@
         <v>1.67</v>
       </c>
       <c r="H1566" t="str">
-        <v>251022QW8WRWC1</v>
+        <v/>
       </c>
       <c r="I1566" t="str">
         <v>money</v>
@@ -74506,7 +74506,7 @@
         <v>30.5</v>
       </c>
       <c r="H1572" t="str">
-        <v>Aleatorio</v>
+        <v/>
       </c>
       <c r="I1572" t="str">
         <v>money</v>
@@ -74535,7 +74535,7 @@
         <v>30.5</v>
       </c>
       <c r="H1573" t="str">
-        <v>2510263XS7F3J5</v>
+        <v/>
       </c>
       <c r="I1573" t="str">
         <v>money</v>
@@ -74564,7 +74564,7 @@
         <v>30.5</v>
       </c>
       <c r="H1574" t="str">
-        <v>2510265F9DN9NR</v>
+        <v/>
       </c>
       <c r="I1574" t="str">
         <v>money</v>
@@ -74593,7 +74593,7 @@
         <v>30.5</v>
       </c>
       <c r="H1575" t="str">
-        <v>2510265HBSHQD7</v>
+        <v/>
       </c>
       <c r="I1575" t="str">
         <v>money</v>
@@ -74622,7 +74622,7 @@
         <v>102.1</v>
       </c>
       <c r="H1576" t="str">
-        <v>2510276H79S327</v>
+        <v/>
       </c>
       <c r="I1576" t="str">
         <v>money</v>
@@ -74680,7 +74680,7 @@
         <v>22.5</v>
       </c>
       <c r="H1578" t="str">
-        <v>251028AN3589SG</v>
+        <v/>
       </c>
       <c r="I1578" t="str">
         <v>money</v>
@@ -74709,7 +74709,7 @@
         <v>22.5</v>
       </c>
       <c r="H1579" t="str">
-        <v>25102890QMSA50</v>
+        <v/>
       </c>
       <c r="I1579" t="str">
         <v>money</v>
@@ -74767,7 +74767,7 @@
         <v>21.72</v>
       </c>
       <c r="H1581" t="str">
-        <v>251029D5F5A0CC</v>
+        <v/>
       </c>
       <c r="I1581" t="str">
         <v>money</v>
@@ -74796,7 +74796,7 @@
         <v>44.75</v>
       </c>
       <c r="H1582" t="str">
-        <v>251030D9DEWAE9</v>
+        <v/>
       </c>
       <c r="I1582" t="str">
         <v>money</v>
@@ -74825,7 +74825,7 @@
         <v>71.16</v>
       </c>
       <c r="H1583" t="str">
-        <v>251030F8S9STWN</v>
+        <v/>
       </c>
       <c r="I1583" t="str">
         <v>money</v>
@@ -74854,7 +74854,7 @@
         <v>21.72</v>
       </c>
       <c r="H1584" t="str">
-        <v>251029D5F5A0CC</v>
+        <v/>
       </c>
       <c r="I1584" t="str">
         <v>money</v>
@@ -74912,7 +74912,7 @@
         <v>3</v>
       </c>
       <c r="H1586" t="str">
-        <v>francisca</v>
+        <v/>
       </c>
       <c r="I1586" t="str">
         <v>money</v>
@@ -74970,7 +74970,7 @@
         <v>34.9</v>
       </c>
       <c r="H1588" t="str">
-        <v>251102NJ6SPH85</v>
+        <v/>
       </c>
       <c r="I1588" t="str">
         <v>money</v>
@@ -74999,7 +74999,7 @@
         <v>40</v>
       </c>
       <c r="H1589" t="str">
-        <v>251102Q652RSH7</v>
+        <v/>
       </c>
       <c r="I1589" t="str">
         <v>money</v>
@@ -75028,7 +75028,7 @@
         <v>33.37</v>
       </c>
       <c r="H1590" t="str">
-        <v>251102MYQY566D</v>
+        <v/>
       </c>
       <c r="I1590" t="str">
         <v>money</v>
@@ -75057,7 +75057,7 @@
         <v>3.74</v>
       </c>
       <c r="H1591" t="str">
-        <v>251103SHJAKJES</v>
+        <v/>
       </c>
       <c r="I1591" t="str">
         <v>money</v>
@@ -75115,7 +75115,7 @@
         <v>1.71</v>
       </c>
       <c r="H1593" t="str">
-        <v>evandrodo206</v>
+        <v/>
       </c>
       <c r="I1593" t="str">
         <v>money</v>
@@ -75144,7 +75144,7 @@
         <v>33.37</v>
       </c>
       <c r="H1594" t="str">
-        <v>evandrodo206</v>
+        <v/>
       </c>
       <c r="I1594" t="str">
         <v>money</v>
@@ -75173,7 +75173,7 @@
         <v>34.9</v>
       </c>
       <c r="H1595" t="str">
-        <v>fj5laf_w9t</v>
+        <v/>
       </c>
       <c r="I1595" t="str">
         <v>money</v>
@@ -75231,7 +75231,7 @@
         <v>32</v>
       </c>
       <c r="H1597" t="str">
-        <v>zelton.novais</v>
+        <v/>
       </c>
       <c r="I1597" t="str">
         <v>money</v>
@@ -75405,7 +75405,7 @@
         <v>0</v>
       </c>
       <c r="H1603" t="str">
-        <v>Aleatorio</v>
+        <v/>
       </c>
       <c r="I1603" t="str">
         <v>money</v>
@@ -75434,7 +75434,7 @@
         <v>98.12</v>
       </c>
       <c r="H1604" t="str">
-        <v>Aleatorio</v>
+        <v/>
       </c>
       <c r="I1604" t="str">
         <v>money</v>
@@ -76855,7 +76855,7 @@
         <v>6.3</v>
       </c>
       <c r="H1653" t="str">
-        <v>251125N6D00GHN</v>
+        <v/>
       </c>
       <c r="I1653" t="str">
         <v>money</v>
@@ -76884,7 +76884,7 @@
         <v>6.3</v>
       </c>
       <c r="H1654" t="str">
-        <v>251126QTAS3SAR</v>
+        <v/>
       </c>
       <c r="I1654" t="str">
         <v>money</v>
@@ -76913,7 +76913,7 @@
         <v>34</v>
       </c>
       <c r="H1655" t="str">
-        <v>2511195SVS58WQ</v>
+        <v/>
       </c>
       <c r="I1655" t="str">
         <v>money</v>
@@ -77145,7 +77145,7 @@
         <v>21</v>
       </c>
       <c r="H1663" t="str">
-        <v>251127T0EUU1WM</v>
+        <v/>
       </c>
       <c r="I1663" t="str">
         <v>money</v>
@@ -77174,7 +77174,7 @@
         <v>77.88</v>
       </c>
       <c r="H1664" t="str">
-        <v>7550209518518535943</v>
+        <v/>
       </c>
       <c r="I1664" t="str">
         <v>money</v>
@@ -77667,7 +77667,7 @@
         <v>4</v>
       </c>
       <c r="H1681" t="str">
-        <v>2512016D13CT6U</v>
+        <v/>
       </c>
       <c r="I1681" t="str">
         <v>money</v>
@@ -77696,7 +77696,7 @@
         <v>84</v>
       </c>
       <c r="H1682" t="str">
-        <v>251204E2WQ3CR3</v>
+        <v/>
       </c>
       <c r="I1682" t="str">
         <v>money</v>
@@ -77725,7 +77725,7 @@
         <v>21</v>
       </c>
       <c r="H1683" t="str">
-        <v>25112819EYDS0J</v>
+        <v/>
       </c>
       <c r="I1683" t="str">
         <v>money</v>
@@ -77754,7 +77754,7 @@
         <v>30.24</v>
       </c>
       <c r="H1684" t="str">
-        <v>251208S746WPVS</v>
+        <v/>
       </c>
       <c r="I1684" t="str">
         <v>money</v>
@@ -77783,7 +77783,7 @@
         <v>9</v>
       </c>
       <c r="H1685" t="str">
-        <v>251208TBTU0JQX</v>
+        <v/>
       </c>
       <c r="I1685" t="str">
         <v>money</v>
@@ -77812,7 +77812,7 @@
         <v>30.24</v>
       </c>
       <c r="H1686" t="str">
-        <v>251208RNR5ABPX</v>
+        <v/>
       </c>
       <c r="I1686" t="str">
         <v>money</v>
@@ -77841,7 +77841,7 @@
         <v>30.24</v>
       </c>
       <c r="H1687" t="str">
-        <v>251206KWK4SX80</v>
+        <v/>
       </c>
       <c r="I1687" t="str">
         <v>money</v>
@@ -77870,7 +77870,7 @@
         <v>30.24</v>
       </c>
       <c r="H1688" t="str">
-        <v>251205JU4D091G</v>
+        <v/>
       </c>
       <c r="I1688" t="str">
         <v>money</v>
@@ -77899,7 +77899,7 @@
         <v>21</v>
       </c>
       <c r="H1689" t="str">
-        <v>251127T0EUU1WM</v>
+        <v/>
       </c>
       <c r="I1689" t="str">
         <v>money</v>
@@ -77928,7 +77928,7 @@
         <v>10.74</v>
       </c>
       <c r="H1690" t="str">
-        <v>25112811QMV818</v>
+        <v/>
       </c>
       <c r="I1690" t="str">
         <v>money</v>
@@ -77957,7 +77957,7 @@
         <v>4.24</v>
       </c>
       <c r="H1691" t="str">
-        <v>251204E6UDR503</v>
+        <v/>
       </c>
       <c r="I1691" t="str">
         <v>money</v>
@@ -77986,7 +77986,7 @@
         <v>11.74</v>
       </c>
       <c r="H1692" t="str">
-        <v>251204EPGA4ETC</v>
+        <v/>
       </c>
       <c r="I1692" t="str">
         <v>money</v>
@@ -78015,7 +78015,7 @@
         <v>6.3</v>
       </c>
       <c r="H1693" t="str">
-        <v>251205GCHYG20G</v>
+        <v/>
       </c>
       <c r="I1693" t="str">
         <v>money</v>
@@ -78044,7 +78044,7 @@
         <v>21</v>
       </c>
       <c r="H1694" t="str">
-        <v>251205HE7YTHM6</v>
+        <v/>
       </c>
       <c r="I1694" t="str">
         <v>money</v>
@@ -78073,7 +78073,7 @@
         <v>7.63</v>
       </c>
       <c r="H1695" t="str">
-        <v>251208SMPRG11A</v>
+        <v/>
       </c>
       <c r="I1695" t="str">
         <v>money</v>
@@ -78102,7 +78102,7 @@
         <v>6.3</v>
       </c>
       <c r="H1696" t="str">
-        <v>251208R3JYP1TD</v>
+        <v/>
       </c>
       <c r="I1696" t="str">
         <v>money</v>
@@ -78131,7 +78131,7 @@
         <v>1.43</v>
       </c>
       <c r="H1697" t="str">
-        <v>251207QQBN0Q1H</v>
+        <v/>
       </c>
       <c r="I1697" t="str">
         <v>money</v>
@@ -78160,7 +78160,7 @@
         <v>19</v>
       </c>
       <c r="H1698" t="str">
-        <v>Aleatorio</v>
+        <v/>
       </c>
       <c r="I1698" t="str">
         <v>money</v>
@@ -78653,7 +78653,7 @@
         <v>270</v>
       </c>
       <c r="H1715" t="str">
-        <v>Aleatorio</v>
+        <v/>
       </c>
       <c r="I1715" t="str">
         <v>money</v>
@@ -79233,7 +79233,7 @@
         <v>153</v>
       </c>
       <c r="H1735" t="str">
-        <v>251217JA47THQU</v>
+        <v/>
       </c>
       <c r="I1735" t="str">
         <v>money</v>
@@ -79262,7 +79262,7 @@
         <v>105</v>
       </c>
       <c r="H1736" t="str">
-        <v>1733237725498345439</v>
+        <v/>
       </c>
       <c r="I1736" t="str">
         <v>money</v>
@@ -79407,7 +79407,7 @@
         <v>258</v>
       </c>
       <c r="H1741" t="str">
-        <v>581764922242532626</v>
+        <v/>
       </c>
       <c r="I1741" t="str">
         <v>money</v>
@@ -79871,7 +79871,7 @@
         <v>30.24</v>
       </c>
       <c r="H1757" t="str">
-        <v>251226BB55U3C7</v>
+        <v/>
       </c>
       <c r="I1757" t="str">
         <v>money</v>
@@ -79900,7 +79900,7 @@
         <v>30.24</v>
       </c>
       <c r="H1758" t="str">
-        <v>251228GM6DF9FD</v>
+        <v/>
       </c>
       <c r="I1758" t="str">
         <v>money</v>
@@ -79929,7 +79929,7 @@
         <v>8.5</v>
       </c>
       <c r="H1759" t="str">
-        <v>251228GQAC35RE</v>
+        <v/>
       </c>
       <c r="I1759" t="str">
         <v>money</v>
@@ -80103,7 +80103,7 @@
         <v>98.4</v>
       </c>
       <c r="H1765" t="str">
-        <v>581881466757613048</v>
+        <v/>
       </c>
       <c r="I1765" t="str">
         <v>money</v>
@@ -80190,7 +80190,7 @@
         <v>41.2</v>
       </c>
       <c r="H1768" t="str">
-        <v>26010470HA378U</v>
+        <v/>
       </c>
       <c r="I1768" t="str">
         <v>pix</v>
@@ -80219,7 +80219,7 @@
         <v>26.6</v>
       </c>
       <c r="H1769" t="str">
-        <v>2601057PDHKMGS</v>
+        <v/>
       </c>
       <c r="I1769" t="str">
         <v>pix</v>
@@ -80248,7 +80248,7 @@
         <v>2.99</v>
       </c>
       <c r="H1770" t="str">
-        <v>26010322KX6CM7</v>
+        <v/>
       </c>
       <c r="I1770" t="str">
         <v>pix</v>
@@ -80277,7 +80277,7 @@
         <v>2.99</v>
       </c>
       <c r="H1771" t="str">
-        <v>26010321EYMMGF</v>
+        <v/>
       </c>
       <c r="I1771" t="str">
         <v>pix</v>
@@ -80306,7 +80306,7 @@
         <v>15.75</v>
       </c>
       <c r="H1772" t="str">
-        <v>26010330Y0QYCC</v>
+        <v/>
       </c>
       <c r="I1772" t="str">
         <v>pix</v>
@@ -80596,7 +80596,7 @@
         <v>13.1</v>
       </c>
       <c r="H1782" t="str">
-        <v>260113UN53PDB3</v>
+        <v/>
       </c>
       <c r="I1782" t="str">
         <v>pix</v>
@@ -80625,7 +80625,7 @@
         <v>100.32</v>
       </c>
       <c r="H1783" t="str">
-        <v>1732942733137053663</v>
+        <v/>
       </c>
       <c r="I1783" t="str">
         <v>pix</v>
@@ -80712,7 +80712,7 @@
         <v>1.54</v>
       </c>
       <c r="H1786" t="str">
-        <v>26011533GTJVCC</v>
+        <v/>
       </c>
       <c r="I1786" t="str">
         <v>pix</v>
@@ -80741,7 +80741,7 @@
         <v>27.99</v>
       </c>
       <c r="H1787" t="str">
-        <v>260115363HXRNS</v>
+        <v/>
       </c>
       <c r="I1787" t="str">
         <v>pix</v>
@@ -81437,7 +81437,7 @@
         <v>3.7</v>
       </c>
       <c r="H1811" t="str">
-        <v>260120HKJW21F6</v>
+        <v/>
       </c>
       <c r="I1811" t="str">
         <v>pix</v>
@@ -81466,7 +81466,7 @@
         <v>45.84</v>
       </c>
       <c r="H1812" t="str">
-        <v>260120HW0K4N7G</v>
+        <v/>
       </c>
       <c r="I1812" t="str">
         <v>pix</v>
@@ -81727,7 +81727,7 @@
         <v>5.56</v>
       </c>
       <c r="H1821" t="str">
-        <v>26012501R0305B</v>
+        <v/>
       </c>
       <c r="I1821" t="str">
         <v>pix</v>
@@ -81756,7 +81756,7 @@
         <v>3.46</v>
       </c>
       <c r="H1822" t="str">
-        <v>260125W10MYBA6</v>
+        <v/>
       </c>
       <c r="I1822" t="str">
         <v>pix</v>
@@ -81785,7 +81785,7 @@
         <v>12.56</v>
       </c>
       <c r="H1823" t="str">
-        <v>260123QKXEPFNT</v>
+        <v/>
       </c>
       <c r="I1823" t="str">
         <v>pix</v>
@@ -81814,7 +81814,7 @@
         <v>38.39</v>
       </c>
       <c r="H1824" t="str">
-        <v>2601262EWM7HSQ</v>
+        <v/>
       </c>
       <c r="I1824" t="str">
         <v>pix</v>
@@ -81843,7 +81843,7 @@
         <v>7.61</v>
       </c>
       <c r="H1825" t="str">
-        <v>26012643AWWXYN</v>
+        <v/>
       </c>
       <c r="I1825" t="str">
         <v>pix</v>
@@ -81901,7 +81901,7 @@
         <v>6.32</v>
       </c>
       <c r="H1827" t="str">
-        <v>26012877ASXSW2</v>
+        <v/>
       </c>
       <c r="I1827" t="str">
         <v>pix</v>
@@ -81930,7 +81930,7 @@
         <v>6.32</v>
       </c>
       <c r="H1828" t="str">
-        <v>26012879CE069S</v>
+        <v/>
       </c>
       <c r="I1828" t="str">
         <v>pix</v>
@@ -81959,7 +81959,7 @@
         <v>6.54</v>
       </c>
       <c r="H1829" t="str">
-        <v>2601287HCSF395</v>
+        <v/>
       </c>
       <c r="I1829" t="str">
         <v>pix</v>
@@ -81988,7 +81988,7 @@
         <v>6.32</v>
       </c>
       <c r="H1830" t="str">
-        <v>2601288URC8VEF</v>
+        <v/>
       </c>
       <c r="I1830" t="str">
         <v>pix</v>
@@ -82104,7 +82104,7 @@
         <v>45.39</v>
       </c>
       <c r="H1834" t="str">
-        <v>260131E6UQ7MER</v>
+        <v/>
       </c>
       <c r="I1834" t="str">
         <v>pix</v>
@@ -82162,7 +82162,7 @@
         <v>55.2</v>
       </c>
       <c r="H1836" t="str">
-        <v>582355031501800714</v>
+        <v/>
       </c>
       <c r="I1836" t="str">
         <v>pix</v>
@@ -82278,7 +82278,7 @@
         <v>63.96</v>
       </c>
       <c r="H1840" t="str">
-        <v>260202KGB8PW0S</v>
+        <v/>
       </c>
       <c r="I1840" t="str">
         <v>pix</v>
@@ -82307,7 +82307,7 @@
         <v>6.32</v>
       </c>
       <c r="H1841" t="str">
-        <v>260202KDJAYA04</v>
+        <v/>
       </c>
       <c r="I1841" t="str">
         <v>pix</v>
@@ -82336,7 +82336,7 @@
         <v>6.32</v>
       </c>
       <c r="H1842" t="str">
-        <v>260202KB9XFY1F</v>
+        <v/>
       </c>
       <c r="I1842" t="str">
         <v>pix</v>
@@ -82365,7 +82365,7 @@
         <v>28.58</v>
       </c>
       <c r="H1843" t="str">
-        <v>260201HUCC9A14</v>
+        <v/>
       </c>
       <c r="I1843" t="str">
         <v>pix</v>
@@ -82394,7 +82394,7 @@
         <v>6.54</v>
       </c>
       <c r="H1844" t="str">
-        <v>260130BPA5UXQ0</v>
+        <v/>
       </c>
       <c r="I1844" t="str">
         <v>pix</v>
@@ -82481,7 +82481,7 @@
         <v>6.79</v>
       </c>
       <c r="H1847" t="str">
-        <v>260203QVC1NHGG</v>
+        <v/>
       </c>
       <c r="I1847" t="str">
         <v>pix</v>
@@ -82510,7 +82510,7 @@
         <v>6.32</v>
       </c>
       <c r="H1848" t="str">
-        <v>260203PK6Y0A25</v>
+        <v/>
       </c>
       <c r="I1848" t="str">
         <v>pix</v>
@@ -82539,7 +82539,7 @@
         <v>6.5</v>
       </c>
       <c r="H1849" t="str">
-        <v>260203PRHGUC97</v>
+        <v/>
       </c>
       <c r="I1849" t="str">
         <v>pix</v>
@@ -82568,7 +82568,7 @@
         <v>7.49</v>
       </c>
       <c r="H1850" t="str">
-        <v>260203Q3C34DNC</v>
+        <v/>
       </c>
       <c r="I1850" t="str">
         <v>pix</v>
@@ -82597,7 +82597,7 @@
         <v>6.54</v>
       </c>
       <c r="H1851" t="str">
-        <v>260203QJNTUWSC</v>
+        <v/>
       </c>
       <c r="I1851" t="str">
         <v>pix</v>
@@ -82655,7 +82655,7 @@
         <v>6.29</v>
       </c>
       <c r="H1853" t="str">
-        <v>260205TXSABCRN</v>
+        <v/>
       </c>
       <c r="I1853" t="str">
         <v>pix</v>
@@ -82684,7 +82684,7 @@
         <v>6.32</v>
       </c>
       <c r="H1854" t="str">
-        <v>260205TXVP1P5N</v>
+        <v/>
       </c>
       <c r="I1854" t="str">
         <v>pix</v>
@@ -82800,7 +82800,7 @@
         <v>6.32</v>
       </c>
       <c r="H1858" t="str">
-        <v>260205UK2H546J</v>
+        <v/>
       </c>
       <c r="I1858" t="str">
         <v>pix</v>
@@ -82829,7 +82829,7 @@
         <v>6.32</v>
       </c>
       <c r="H1859" t="str">
-        <v>2602060TRY2SPR</v>
+        <v/>
       </c>
       <c r="I1859" t="str">
         <v>pix</v>
@@ -82858,7 +82858,7 @@
         <v>6.32</v>
       </c>
       <c r="H1860" t="str">
-        <v>26020619R29YC5</v>
+        <v/>
       </c>
       <c r="I1860" t="str">
         <v>pix</v>
@@ -82887,7 +82887,7 @@
         <v>6.32</v>
       </c>
       <c r="H1861" t="str">
-        <v>2602061AFHRWQS</v>
+        <v/>
       </c>
       <c r="I1861" t="str">
         <v>pix</v>
@@ -83032,7 +83032,7 @@
         <v>6.5</v>
       </c>
       <c r="H1866" t="str">
-        <v>2602087DYXN63P</v>
+        <v/>
       </c>
       <c r="I1866" t="str">
         <v>pix</v>
@@ -83061,7 +83061,7 @@
         <v>13.1</v>
       </c>
       <c r="H1867" t="str">
-        <v>26020987RHU086</v>
+        <v/>
       </c>
       <c r="I1867" t="str">
         <v>pix</v>
@@ -83235,7 +83235,7 @@
         <v>6.32</v>
       </c>
       <c r="H1873" t="str">
-        <v>2602098NVFCAP8</v>
+        <v/>
       </c>
       <c r="I1873" t="str">
         <v>pix</v>
@@ -83322,7 +83322,7 @@
         <v>6.29</v>
       </c>
       <c r="H1876" t="str">
-        <v>260211EY108RQH</v>
+        <v/>
       </c>
       <c r="I1876" t="str">
         <v>pix</v>
@@ -83380,7 +83380,7 @@
         <v>6.32</v>
       </c>
       <c r="H1878" t="str">
-        <v>260211EVXGJHUB</v>
+        <v/>
       </c>
       <c r="I1878" t="str">
         <v>pix</v>
@@ -83409,7 +83409,7 @@
         <v>6.32</v>
       </c>
       <c r="H1879" t="str">
-        <v>260212G46PXBNW</v>
+        <v/>
       </c>
       <c r="I1879" t="str">
         <v>pix</v>
@@ -83438,7 +83438,7 @@
         <v>4.64</v>
       </c>
       <c r="H1880" t="str">
-        <v>260212G72M35W6</v>
+        <v/>
       </c>
       <c r="I1880" t="str">
         <v>pix</v>
@@ -83467,7 +83467,7 @@
         <v>13.94</v>
       </c>
       <c r="H1881" t="str">
-        <v>260212G4R2W2EE</v>
+        <v/>
       </c>
       <c r="I1881" t="str">
         <v>pix</v>
@@ -83554,7 +83554,7 @@
         <v>13.02</v>
       </c>
       <c r="H1884" t="str">
-        <v>260213JQR733AV</v>
+        <v/>
       </c>
       <c r="I1884" t="str">
         <v>pix</v>
@@ -83583,7 +83583,7 @@
         <v>6.32</v>
       </c>
       <c r="H1885" t="str">
-        <v>260213JDRSN8HV</v>
+        <v/>
       </c>
       <c r="I1885" t="str">
         <v>pix</v>
@@ -83612,7 +83612,7 @@
         <v>6.32</v>
       </c>
       <c r="H1886" t="str">
-        <v>260213HSDSJMQX</v>
+        <v/>
       </c>
       <c r="I1886" t="str">
         <v>pix</v>
@@ -83699,7 +83699,7 @@
         <v>186.52</v>
       </c>
       <c r="H1889" t="str">
-        <v>260214MX09MKJK</v>
+        <v/>
       </c>
       <c r="I1889" t="str">
         <v>pix</v>
@@ -83786,7 +83786,7 @@
         <v>6.5</v>
       </c>
       <c r="H1892" t="str">
-        <v>260214PRACWP1G</v>
+        <v/>
       </c>
       <c r="I1892" t="str">
         <v>pix</v>
@@ -83815,7 +83815,7 @@
         <v>6.5</v>
       </c>
       <c r="H1893" t="str">
-        <v>260214NC6AV4AW</v>
+        <v/>
       </c>
       <c r="I1893" t="str">
         <v>pix</v>
@@ -83844,7 +83844,7 @@
         <v>6.5</v>
       </c>
       <c r="H1894" t="str">
-        <v>260215S10WG2NV</v>
+        <v/>
       </c>
       <c r="I1894" t="str">
         <v>pix</v>
@@ -83873,7 +83873,7 @@
         <v>6.5</v>
       </c>
       <c r="H1895" t="str">
-        <v>260215QY2AJYYW</v>
+        <v/>
       </c>
       <c r="I1895" t="str">
         <v>pix</v>
@@ -83902,7 +83902,7 @@
         <v>6.5</v>
       </c>
       <c r="H1896" t="str">
-        <v>260215S0NNWVA1</v>
+        <v/>
       </c>
       <c r="I1896" t="str">
         <v>pix</v>
@@ -83931,7 +83931,7 @@
         <v>1.54</v>
       </c>
       <c r="H1897" t="str">
-        <v>260216UC5PEXQS</v>
+        <v/>
       </c>
       <c r="I1897" t="str">
         <v>pix</v>
@@ -83960,7 +83960,7 @@
         <v>4.64</v>
       </c>
       <c r="H1898" t="str">
-        <v>260216T9YQWBCN</v>
+        <v/>
       </c>
       <c r="I1898" t="str">
         <v>pix</v>
@@ -83989,7 +83989,7 @@
         <v>4.8</v>
       </c>
       <c r="H1899" t="str">
-        <v>260216UB0PYHCE</v>
+        <v/>
       </c>
       <c r="I1899" t="str">
         <v>pix</v>
@@ -84047,7 +84047,7 @@
         <v>4.8</v>
       </c>
       <c r="H1901" t="str">
-        <v>2602181G0BWP7K</v>
+        <v/>
       </c>
       <c r="I1901" t="str">
         <v>pix</v>
@@ -84076,7 +84076,7 @@
         <v>4.64</v>
       </c>
       <c r="H1902" t="str">
-        <v>2602170V61Y572</v>
+        <v/>
       </c>
       <c r="I1902" t="str">
         <v>pix</v>
@@ -84221,7 +84221,7 @@
         <v>8.8</v>
       </c>
       <c r="H1907" t="str">
-        <v>2602194QD3PDMR</v>
+        <v/>
       </c>
       <c r="I1907" t="str">
         <v>pix</v>
@@ -84250,7 +84250,7 @@
         <v>6.54</v>
       </c>
       <c r="H1908" t="str">
-        <v>260219506EESHD</v>
+        <v/>
       </c>
       <c r="I1908" t="str">
         <v>pix</v>
@@ -84279,7 +84279,7 @@
         <v>4.8</v>
       </c>
       <c r="H1909" t="str">
-        <v>26022088CEW7MH</v>
+        <v/>
       </c>
       <c r="I1909" t="str">
         <v>pix</v>
@@ -84308,7 +84308,7 @@
         <v>8.29</v>
       </c>
       <c r="H1910" t="str">
-        <v>582671832439162687</v>
+        <v/>
       </c>
       <c r="I1910" t="str">
         <v>pix</v>
@@ -84337,7 +84337,7 @@
         <v>74.2</v>
       </c>
       <c r="H1911" t="str">
-        <v>582693256409416785</v>
+        <v/>
       </c>
       <c r="I1911" t="str">
         <v>pix</v>
@@ -84482,7 +84482,7 @@
         <v>9.3</v>
       </c>
       <c r="H1916" t="str">
-        <v>260223DWGFD4CB</v>
+        <v/>
       </c>
       <c r="I1916" t="str">
         <v>pix</v>
@@ -84511,7 +84511,7 @@
         <v>14.54</v>
       </c>
       <c r="H1917" t="str">
-        <v>260223E5E800MU</v>
+        <v/>
       </c>
       <c r="I1917" t="str">
         <v>pix</v>
@@ -84598,7 +84598,7 @@
         <v>8.5</v>
       </c>
       <c r="H1920" t="str">
-        <v>582767102684267825</v>
+        <v/>
       </c>
       <c r="I1920" t="str">
         <v>pix</v>
@@ -84627,7 +84627,7 @@
         <v>4.8</v>
       </c>
       <c r="H1921" t="str">
-        <v>260224HATE1P51</v>
+        <v/>
       </c>
       <c r="I1921" t="str">
         <v>pix</v>
@@ -84685,7 +84685,7 @@
         <v>17.2</v>
       </c>
       <c r="H1923" t="str">
-        <v>582832973697222108</v>
+        <v/>
       </c>
       <c r="I1923" t="str">
         <v>pix</v>
@@ -84714,7 +84714,7 @@
         <v>8.5</v>
       </c>
       <c r="H1924" t="str">
-        <v>582802201370330561</v>
+        <v/>
       </c>
       <c r="I1924" t="str">
         <v>pix</v>
@@ -85178,7 +85178,7 @@
         <v>150</v>
       </c>
       <c r="H1940" t="str">
-        <v>olx</v>
+        <v/>
       </c>
       <c r="I1940" t="str">
         <v>pix</v>
@@ -85236,7 +85236,7 @@
         <v>8.29</v>
       </c>
       <c r="H1942" t="str">
-        <v>582949664542655793</v>
+        <v/>
       </c>
       <c r="I1942" t="str">
         <v>pix</v>
@@ -85265,7 +85265,7 @@
         <v>16.58</v>
       </c>
       <c r="H1943" t="str">
-        <v>582969363430213371</v>
+        <v/>
       </c>
       <c r="I1943" t="str">
         <v>pix</v>
@@ -85381,7 +85381,7 @@
         <v>6.32</v>
       </c>
       <c r="H1947" t="str">
-        <v>2603143RH3G5SJ</v>
+        <v/>
       </c>
       <c r="I1947" t="str">
         <v>pix</v>
@@ -85410,7 +85410,7 @@
         <v>4.8</v>
       </c>
       <c r="H1948" t="str">
-        <v>260311SUCVJT5B</v>
+        <v/>
       </c>
       <c r="I1948" t="str">
         <v>pix</v>
@@ -85439,7 +85439,7 @@
         <v>4.8</v>
       </c>
       <c r="H1949" t="str">
-        <v>260312UJJBBAVE</v>
+        <v/>
       </c>
       <c r="I1949" t="str">
         <v>pix</v>
@@ -85468,7 +85468,7 @@
         <v>4.8</v>
       </c>
       <c r="H1950" t="str">
-        <v>260311SA40Y1F8</v>
+        <v/>
       </c>
       <c r="I1950" t="str">
         <v>pix</v>
@@ -85497,7 +85497,7 @@
         <v>4.8</v>
       </c>
       <c r="H1951" t="str">
-        <v>260311SNXJHKSB</v>
+        <v/>
       </c>
       <c r="I1951" t="str">
         <v>pix</v>
@@ -85526,7 +85526,7 @@
         <v>4.8</v>
       </c>
       <c r="H1952" t="str">
-        <v>260313103HV5F6</v>
+        <v/>
       </c>
       <c r="I1952" t="str">
         <v>pix</v>
@@ -85555,7 +85555,7 @@
         <v>4.8</v>
       </c>
       <c r="H1953" t="str">
-        <v>2603131G6CJM2Y</v>
+        <v/>
       </c>
       <c r="I1953" t="str">
         <v>pix</v>
@@ -85584,7 +85584,7 @@
         <v>4.8</v>
       </c>
       <c r="H1954" t="str">
-        <v>26031325T58KDX</v>
+        <v/>
       </c>
       <c r="I1954" t="str">
         <v>pix</v>
@@ -85613,7 +85613,7 @@
         <v>4.8</v>
       </c>
       <c r="H1955" t="str">
-        <v>2603143K853WWM</v>
+        <v/>
       </c>
       <c r="I1955" t="str">
         <v>pix</v>
@@ -85642,7 +85642,7 @@
         <v>4.8</v>
       </c>
       <c r="H1956" t="str">
-        <v>2603145F5U847D</v>
+        <v/>
       </c>
       <c r="I1956" t="str">
         <v>pix</v>
@@ -85671,7 +85671,7 @@
         <v>28.52</v>
       </c>
       <c r="H1957" t="str">
-        <v>583003560395768948</v>
+        <v/>
       </c>
       <c r="I1957" t="str">
         <v>pix</v>
@@ -85700,7 +85700,7 @@
         <v>8.29</v>
       </c>
       <c r="H1958" t="str">
-        <v>583028210992842730</v>
+        <v/>
       </c>
       <c r="I1958" t="str">
         <v>pix</v>
@@ -85729,7 +85729,7 @@
         <v>8.29</v>
       </c>
       <c r="H1959" t="str">
-        <v>583076402794039259</v>
+        <v/>
       </c>
       <c r="I1959" t="str">
         <v>pix</v>
@@ -85758,7 +85758,7 @@
         <v>103.69</v>
       </c>
       <c r="H1960" t="str">
-        <v>2603156GA6X2KW</v>
+        <v/>
       </c>
       <c r="I1960" t="str">
         <v>pix</v>
@@ -85787,7 +85787,7 @@
         <v>4.8</v>
       </c>
       <c r="H1961" t="str">
-        <v>2603168MB44W5B</v>
+        <v/>
       </c>
       <c r="I1961" t="str">
         <v>pix</v>
@@ -85816,7 +85816,7 @@
         <v>4.8</v>
       </c>
       <c r="H1962" t="str">
-        <v>2603157YRJQ60Y</v>
+        <v/>
       </c>
       <c r="I1962" t="str">
         <v>pix</v>
@@ -85845,7 +85845,7 @@
         <v>4.8</v>
       </c>
       <c r="H1963" t="str">
-        <v>2603168N84XUJ5</v>
+        <v/>
       </c>
       <c r="I1963" t="str">
         <v>pix</v>
@@ -85874,7 +85874,7 @@
         <v>4.8</v>
       </c>
       <c r="H1964" t="str">
-        <v>2603169878A177</v>
+        <v/>
       </c>
       <c r="I1964" t="str">
         <v>pix</v>
@@ -86048,7 +86048,7 @@
         <v>4.8</v>
       </c>
       <c r="H1970" t="str">
-        <v>260320MRH5UP5A</v>
+        <v/>
       </c>
       <c r="I1970" t="str">
         <v>pix</v>
@@ -86077,7 +86077,7 @@
         <v>6.54</v>
       </c>
       <c r="H1971" t="str">
-        <v>260323UA87XECC</v>
+        <v/>
       </c>
       <c r="I1971" t="str">
         <v>pix</v>
@@ -86164,7 +86164,7 @@
         <v>8.5</v>
       </c>
       <c r="H1974" t="str">
-        <v>583086581104871031</v>
+        <v/>
       </c>
       <c r="I1974" t="str">
         <v>money</v>
@@ -86193,7 +86193,7 @@
         <v>8.29</v>
       </c>
       <c r="H1975" t="str">
-        <v>583098538648110579</v>
+        <v/>
       </c>
       <c r="I1975" t="str">
         <v>money</v>
@@ -86222,7 +86222,7 @@
         <v>8.5</v>
       </c>
       <c r="H1976" t="str">
-        <v>583114960457861054</v>
+        <v/>
       </c>
       <c r="I1976" t="str">
         <v>money</v>
@@ -86251,7 +86251,7 @@
         <v>8.5</v>
       </c>
       <c r="H1977" t="str">
-        <v>583128761118000431</v>
+        <v/>
       </c>
       <c r="I1977" t="str">
         <v>money</v>
@@ -86280,7 +86280,7 @@
         <v>8.29</v>
       </c>
       <c r="H1978" t="str">
-        <v>583128912663119443</v>
+        <v/>
       </c>
       <c r="I1978" t="str">
         <v>money</v>
@@ -86309,7 +86309,7 @@
         <v>8.29</v>
       </c>
       <c r="H1979" t="str">
-        <v>583155029219772144</v>
+        <v/>
       </c>
       <c r="I1979" t="str">
         <v>money</v>
@@ -86338,7 +86338,7 @@
         <v>25.8</v>
       </c>
       <c r="H1980" t="str">
-        <v>583191996668544497</v>
+        <v/>
       </c>
       <c r="I1980" t="str">
         <v>money</v>
@@ -86686,7 +86686,7 @@
         <v>15</v>
       </c>
       <c r="H1992" t="str">
-        <v>2604052N4YAKVP</v>
+        <v/>
       </c>
       <c r="I1992" t="str">
         <v>pix</v>
@@ -86715,7 +86715,7 @@
         <v>4.8</v>
       </c>
       <c r="H1993" t="str">
-        <v>260403U0Q395NK</v>
+        <v/>
       </c>
       <c r="I1993" t="str">
         <v>pix</v>
@@ -86744,7 +86744,7 @@
         <v>4.8</v>
       </c>
       <c r="H1994" t="str">
-        <v>260403TU7QV6XT</v>
+        <v/>
       </c>
       <c r="I1994" t="str">
         <v>pix</v>
@@ -86773,7 +86773,7 @@
         <v>4.8</v>
       </c>
       <c r="H1995" t="str">
-        <v>260401NR0BA272</v>
+        <v/>
       </c>
       <c r="I1995" t="str">
         <v>pix</v>
@@ -86802,7 +86802,7 @@
         <v>4.8</v>
       </c>
       <c r="H1996" t="str">
-        <v>260328BWM81AGS</v>
+        <v/>
       </c>
       <c r="I1996" t="str">
         <v>pix</v>
@@ -86831,7 +86831,7 @@
         <v>4.8</v>
       </c>
       <c r="H1997" t="str">
-        <v>260409CD2W2XJB</v>
+        <v/>
       </c>
       <c r="I1997" t="str">
         <v>pix</v>
@@ -86860,7 +86860,7 @@
         <v>4.8</v>
       </c>
       <c r="H1998" t="str">
-        <v>260409BFX8SS7A</v>
+        <v/>
       </c>
       <c r="I1998" t="str">
         <v>pix</v>
@@ -86889,7 +86889,7 @@
         <v>4.8</v>
       </c>
       <c r="H1999" t="str">
-        <v>260409BSHH7E0Q</v>
+        <v/>
       </c>
       <c r="I1999" t="str">
         <v>pix</v>
@@ -86918,7 +86918,7 @@
         <v>4.8</v>
       </c>
       <c r="H2000" t="str">
-        <v>2604089DYV9NFE</v>
+        <v/>
       </c>
       <c r="I2000" t="str">
         <v>pix</v>
@@ -86947,7 +86947,7 @@
         <v>4.8</v>
       </c>
       <c r="H2001" t="str">
-        <v>2604088H2RCBCG</v>
+        <v/>
       </c>
       <c r="I2001" t="str">
         <v>pix</v>
@@ -86976,7 +86976,7 @@
         <v>4.8</v>
       </c>
       <c r="H2002" t="str">
-        <v>2604088EAMB58S</v>
+        <v/>
       </c>
       <c r="I2002" t="str">
         <v>pix</v>
@@ -87005,7 +87005,7 @@
         <v>4.8</v>
       </c>
       <c r="H2003" t="str">
-        <v>26040888X1M69H</v>
+        <v/>
       </c>
       <c r="I2003" t="str">
         <v>pix</v>
@@ -87034,7 +87034,7 @@
         <v>4.64</v>
       </c>
       <c r="H2004" t="str">
-        <v>2604088WQH4MP3</v>
+        <v/>
       </c>
       <c r="I2004" t="str">
         <v>pix</v>
@@ -87063,7 +87063,7 @@
         <v>4.64</v>
       </c>
       <c r="H2005" t="str">
-        <v>2604077VFTMCCS</v>
+        <v/>
       </c>
       <c r="I2005" t="str">
         <v>pix</v>
@@ -87092,7 +87092,7 @@
         <v>8.5</v>
       </c>
       <c r="H2006" t="str">
-        <v>583421944481809850</v>
+        <v/>
       </c>
       <c r="I2006" t="str">
         <v>money</v>
@@ -87121,7 +87121,7 @@
         <v>8.5</v>
       </c>
       <c r="H2007" t="str">
-        <v>583435469169263884</v>
+        <v/>
       </c>
       <c r="I2007" t="str">
         <v>money</v>
@@ -87150,7 +87150,7 @@
         <v>8.5</v>
       </c>
       <c r="H2008" t="str">
-        <v>583436730013615732</v>
+        <v/>
       </c>
       <c r="I2008" t="str">
         <v>money</v>
@@ -87237,7 +87237,7 @@
         <v>4.8</v>
       </c>
       <c r="H2011" t="str">
-        <v>260410DK38AXXA</v>
+        <v/>
       </c>
       <c r="I2011" t="str">
         <v>pix</v>
@@ -87266,7 +87266,7 @@
         <v>4.8</v>
       </c>
       <c r="H2012" t="str">
-        <v>260410DP6H17MK</v>
+        <v/>
       </c>
       <c r="I2012" t="str">
         <v>pix</v>
@@ -87295,7 +87295,7 @@
         <v>4.8</v>
       </c>
       <c r="H2013" t="str">
-        <v>260410F789WW11</v>
+        <v/>
       </c>
       <c r="I2013" t="str">
         <v>pix</v>
@@ -87440,7 +87440,7 @@
         <v>23.3</v>
       </c>
       <c r="H2018" t="str">
-        <v>260413PV0SU306</v>
+        <v/>
       </c>
       <c r="I2018" t="str">
         <v>pix</v>
@@ -87469,7 +87469,7 @@
         <v>4.8</v>
       </c>
       <c r="H2019" t="str">
-        <v>260411HKY18FYT</v>
+        <v/>
       </c>
       <c r="I2019" t="str">
         <v>pix</v>
@@ -87498,7 +87498,7 @@
         <v>4.8</v>
       </c>
       <c r="H2020" t="str">
-        <v>260401NR0BA272</v>
+        <v/>
       </c>
       <c r="I2020" t="str">
         <v>pix</v>
@@ -87527,7 +87527,7 @@
         <v>14.1</v>
       </c>
       <c r="H2021" t="str">
-        <v>260413NCR54MQE</v>
+        <v/>
       </c>
       <c r="I2021" t="str">
         <v>pix</v>
@@ -87556,7 +87556,7 @@
         <v>64.33</v>
       </c>
       <c r="H2022" t="str">
-        <v>260414R65317J0</v>
+        <v/>
       </c>
       <c r="I2022" t="str">
         <v>pix</v>
@@ -87585,7 +87585,7 @@
         <v>4.8</v>
       </c>
       <c r="H2023" t="str">
-        <v>260411G5FBQ3XV</v>
+        <v/>
       </c>
       <c r="I2023" t="str">
         <v>pix</v>
@@ -87614,7 +87614,7 @@
         <v>4.8</v>
       </c>
       <c r="H2024" t="str">
-        <v>260411GFJ31RRA</v>
+        <v/>
       </c>
       <c r="I2024" t="str">
         <v>pix</v>
@@ -87643,7 +87643,7 @@
         <v>4.8</v>
       </c>
       <c r="H2025" t="str">
-        <v>260412JPXBAC7T</v>
+        <v/>
       </c>
       <c r="I2025" t="str">
         <v>pix</v>
@@ -87672,7 +87672,7 @@
         <v>4.8</v>
       </c>
       <c r="H2026" t="str">
-        <v>260413MR5QNNP9</v>
+        <v/>
       </c>
       <c r="I2026" t="str">
         <v>pix</v>
@@ -87701,7 +87701,7 @@
         <v>4.8</v>
       </c>
       <c r="H2027" t="str">
-        <v>260412K9E3GT7K</v>
+        <v/>
       </c>
       <c r="I2027" t="str">
         <v>pix</v>
@@ -87730,7 +87730,7 @@
         <v>4.8</v>
       </c>
       <c r="H2028" t="str">
-        <v>260413NHDG2M9S</v>
+        <v/>
       </c>
       <c r="I2028" t="str">
         <v>pix</v>
@@ -87759,7 +87759,7 @@
         <v>8.22</v>
       </c>
       <c r="H2029" t="str">
-        <v>260412KUNPAFPG</v>
+        <v/>
       </c>
       <c r="I2029" t="str">
         <v>pix</v>
@@ -87788,7 +87788,7 @@
         <v>4.8</v>
       </c>
       <c r="H2030" t="str">
-        <v>260413NQ1NXHYE</v>
+        <v/>
       </c>
       <c r="I2030" t="str">
         <v>pix</v>
@@ -87817,7 +87817,7 @@
         <v>4.8</v>
       </c>
       <c r="H2031" t="str">
-        <v>260413PVYRRD3C</v>
+        <v/>
       </c>
       <c r="I2031" t="str">
         <v>pix</v>
@@ -87846,7 +87846,7 @@
         <v>4.8</v>
       </c>
       <c r="H2032" t="str">
-        <v>260415SNH97YP2</v>
+        <v/>
       </c>
       <c r="I2032" t="str">
         <v>pix</v>
@@ -87875,7 +87875,7 @@
         <v>7.88</v>
       </c>
       <c r="H2033" t="str">
-        <v>260414Q9STB3DN</v>
+        <v/>
       </c>
       <c r="I2033" t="str">
         <v>pix</v>
@@ -87904,7 +87904,7 @@
         <v>4.8</v>
       </c>
       <c r="H2034" t="str">
-        <v>260414QVW70J9K</v>
+        <v/>
       </c>
       <c r="I2034" t="str">
         <v>pix</v>
@@ -87933,7 +87933,7 @@
         <v>4.8</v>
       </c>
       <c r="H2035" t="str">
-        <v>2604172JHMVSDW</v>
+        <v/>
       </c>
       <c r="I2035" t="str">
         <v>pix</v>
@@ -87962,7 +87962,7 @@
         <v>4.8</v>
       </c>
       <c r="H2036" t="str">
-        <v>26041847PHYC32</v>
+        <v/>
       </c>
       <c r="I2036" t="str">
         <v>pix</v>
@@ -87991,7 +87991,7 @@
         <v>7.88</v>
       </c>
       <c r="H2037" t="str">
-        <v>26041619KGDYFH</v>
+        <v/>
       </c>
       <c r="I2037" t="str">
         <v>pix</v>
@@ -88020,7 +88020,7 @@
         <v>4.8</v>
       </c>
       <c r="H2038" t="str">
-        <v>2604184UTQHWTB</v>
+        <v/>
       </c>
       <c r="I2038" t="str">
         <v>pix</v>
@@ -88107,7 +88107,7 @@
         <v>8.5</v>
       </c>
       <c r="H2041" t="str">
-        <v>583479030878472056</v>
+        <v/>
       </c>
       <c r="I2041" t="str">
         <v>money</v>
@@ -88136,7 +88136,7 @@
         <v>8.5</v>
       </c>
       <c r="H2042" t="str">
-        <v>583479882090972614</v>
+        <v/>
       </c>
       <c r="I2042" t="str">
         <v>money</v>
@@ -88165,7 +88165,7 @@
         <v>8.5</v>
       </c>
       <c r="H2043" t="str">
-        <v>583496655317993267</v>
+        <v/>
       </c>
       <c r="I2043" t="str">
         <v>money</v>
@@ -88194,7 +88194,7 @@
         <v>25.5</v>
       </c>
       <c r="H2044" t="str">
-        <v>583507949532579537</v>
+        <v/>
       </c>
       <c r="I2044" t="str">
         <v>money</v>
@@ -88223,7 +88223,7 @@
         <v>8.5</v>
       </c>
       <c r="H2045" t="str">
-        <v>583508537126847701</v>
+        <v/>
       </c>
       <c r="I2045" t="str">
         <v>money</v>
@@ -88252,7 +88252,7 @@
         <v>8.5</v>
       </c>
       <c r="H2046" t="str">
-        <v>583535071876711979</v>
+        <v/>
       </c>
       <c r="I2046" t="str">
         <v>money</v>
@@ -88281,7 +88281,7 @@
         <v>8.5</v>
       </c>
       <c r="H2047" t="str">
-        <v>583549454049118089</v>
+        <v/>
       </c>
       <c r="I2047" t="str">
         <v>pix</v>
@@ -88310,7 +88310,7 @@
         <v>17</v>
       </c>
       <c r="H2048" t="str">
-        <v>583551026406720705</v>
+        <v/>
       </c>
       <c r="I2048" t="str">
         <v>money</v>
@@ -88339,7 +88339,7 @@
         <v>8.5</v>
       </c>
       <c r="H2049" t="str">
-        <v>583553405403694455</v>
+        <v/>
       </c>
       <c r="I2049" t="str">
         <v>money</v>
@@ -88484,7 +88484,7 @@
         <v>46.4</v>
       </c>
       <c r="H2054" t="str">
-        <v>260421C6SSPHA5</v>
+        <v/>
       </c>
       <c r="I2054" t="str">
         <v>pix</v>
@@ -88513,7 +88513,7 @@
         <v>46.4</v>
       </c>
       <c r="H2055" t="str">
-        <v>260421CMEX7DWT</v>
+        <v/>
       </c>
       <c r="I2055" t="str">
         <v>pix</v>
@@ -88542,7 +88542,7 @@
         <v>42.29</v>
       </c>
       <c r="H2056" t="str">
-        <v>260421CNENTYWD</v>
+        <v/>
       </c>
       <c r="I2056" t="str">
         <v>pix</v>
@@ -88571,7 +88571,7 @@
         <v>4.8</v>
       </c>
       <c r="H2057" t="str">
-        <v>260421C89S5NE6</v>
+        <v/>
       </c>
       <c r="I2057" t="str">
         <v>pix</v>
@@ -88600,7 +88600,7 @@
         <v>4.8</v>
       </c>
       <c r="H2058" t="str">
-        <v>2604209HXS1DJ5</v>
+        <v/>
       </c>
       <c r="I2058" t="str">
         <v>pix</v>
@@ -88629,7 +88629,7 @@
         <v>4.8</v>
       </c>
       <c r="H2059" t="str">
-        <v>260420BBSM223J</v>
+        <v/>
       </c>
       <c r="I2059" t="str">
         <v>pix</v>
@@ -88948,7 +88948,7 @@
         <v>8.43</v>
       </c>
       <c r="H2070" t="str">
-        <v>2604280T01SJ8T</v>
+        <v/>
       </c>
       <c r="I2070" t="str">
         <v>pix</v>
@@ -88977,7 +88977,7 @@
         <v>38.2</v>
       </c>
       <c r="H2071" t="str">
-        <v>260423K0DD8TQ5</v>
+        <v/>
       </c>
       <c r="I2071" t="str">
         <v>pix</v>
@@ -89006,7 +89006,7 @@
         <v>3.49</v>
       </c>
       <c r="H2072" t="str">
-        <v>260425NRMJTJ1W</v>
+        <v/>
       </c>
       <c r="I2072" t="str">
         <v>pix</v>
@@ -89035,7 +89035,7 @@
         <v>8.43</v>
       </c>
       <c r="H2073" t="str">
-        <v>260426RJS23MB2</v>
+        <v/>
       </c>
       <c r="I2073" t="str">
         <v>pix</v>
@@ -89064,7 +89064,7 @@
         <v>8.43</v>
       </c>
       <c r="H2074" t="str">
-        <v>260426S0SH02BJ</v>
+        <v/>
       </c>
       <c r="I2074" t="str">
         <v>pix</v>
@@ -89093,7 +89093,7 @@
         <v>8.43</v>
       </c>
       <c r="H2075" t="str">
-        <v>2605019WWE8B9Y</v>
+        <v/>
       </c>
       <c r="I2075" t="str">
         <v>pix</v>
@@ -89122,7 +89122,7 @@
         <v>8.43</v>
       </c>
       <c r="H2076" t="str">
-        <v>60502AD1TAKX0</v>
+        <v/>
       </c>
       <c r="I2076" t="str">
         <v>pix</v>
@@ -89151,7 +89151,7 @@
         <v>6.3</v>
       </c>
       <c r="H2077" t="str">
-        <v>260502B264YRW1</v>
+        <v/>
       </c>
       <c r="I2077" t="str">
         <v>pix</v>
@@ -89180,7 +89180,7 @@
         <v>6.3</v>
       </c>
       <c r="H2078" t="str">
-        <v>26042701X1MQWY</v>
+        <v/>
       </c>
       <c r="I2078" t="str">
         <v>pix</v>
@@ -89209,7 +89209,7 @@
         <v>8.43</v>
       </c>
       <c r="H2079" t="str">
-        <v>260505JFA3YXQE</v>
+        <v/>
       </c>
       <c r="I2079" t="str">
         <v>pix</v>
@@ -89238,7 +89238,7 @@
         <v>8.43</v>
       </c>
       <c r="H2080" t="str">
-        <v>260506MDXPYT4P</v>
+        <v/>
       </c>
       <c r="I2080" t="str">
         <v>pix</v>
@@ -89267,7 +89267,7 @@
         <v>8.43</v>
       </c>
       <c r="H2081" t="str">
-        <v>260506MUHE6AAR</v>
+        <v/>
       </c>
       <c r="I2081" t="str">
         <v>pix</v>
@@ -89325,7 +89325,7 @@
         <v>8.5</v>
       </c>
       <c r="H2083" t="str">
-        <v>583876539229374042</v>
+        <v/>
       </c>
       <c r="I2083" t="str">
         <v>money</v>
@@ -89354,7 +89354,7 @@
         <v>3.23</v>
       </c>
       <c r="H2084" t="str">
-        <v>583899379960350386</v>
+        <v/>
       </c>
       <c r="I2084" t="str">
         <v>money</v>
@@ -89383,7 +89383,7 @@
         <v>8.5</v>
       </c>
       <c r="H2085" t="str">
-        <v>583915753558738499</v>
+        <v/>
       </c>
       <c r="I2085" t="str">
         <v>money</v>
@@ -89412,7 +89412,7 @@
         <v>8.5</v>
       </c>
       <c r="H2086" t="str">
-        <v>583619328241861914</v>
+        <v/>
       </c>
       <c r="I2086" t="str">
         <v>money</v>
@@ -89441,7 +89441,7 @@
         <v>24.34</v>
       </c>
       <c r="H2087" t="str">
-        <v>583637996265834144</v>
+        <v/>
       </c>
       <c r="I2087" t="str">
         <v>money</v>
@@ -89470,7 +89470,7 @@
         <v>8.5</v>
       </c>
       <c r="H2088" t="str">
-        <v>583657289674360718</v>
+        <v/>
       </c>
       <c r="I2088" t="str">
         <v>money</v>
@@ -89499,7 +89499,7 @@
         <v>33.54</v>
       </c>
       <c r="H2089" t="str">
-        <v>583699368798159949</v>
+        <v/>
       </c>
       <c r="I2089" t="str">
         <v>money</v>
@@ -89528,7 +89528,7 @@
         <v>8.5</v>
       </c>
       <c r="H2090" t="str">
-        <v>583729687816472455</v>
+        <v/>
       </c>
       <c r="I2090" t="str">
         <v>money</v>
@@ -89557,7 +89557,7 @@
         <v>8.5</v>
       </c>
       <c r="H2091" t="str">
-        <v>583847449511429402</v>
+        <v/>
       </c>
       <c r="I2091" t="str">
         <v>money</v>
@@ -89586,7 +89586,7 @@
         <v>7.48</v>
       </c>
       <c r="H2092" t="str">
-        <v>260507QWTJATPX</v>
+        <v/>
       </c>
       <c r="I2092" t="str">
         <v>pix</v>
@@ -89615,7 +89615,7 @@
         <v>63.02</v>
       </c>
       <c r="H2093" t="str">
-        <v>260507RR9X6HP4</v>
+        <v/>
       </c>
       <c r="I2093" t="str">
         <v>pix</v>
@@ -89789,7 +89789,7 @@
         <v>38.2</v>
       </c>
       <c r="H2099" t="str">
-        <v>260513951BNUXD</v>
+        <v/>
       </c>
       <c r="I2099" t="str">
         <v>pix</v>
@@ -89818,7 +89818,7 @@
         <v>63.02</v>
       </c>
       <c r="H2100" t="str">
-        <v>2605126P91C4RV</v>
+        <v/>
       </c>
       <c r="I2100" t="str">
         <v>pix</v>
@@ -89847,7 +89847,7 @@
         <v>8.43</v>
       </c>
       <c r="H2101" t="str">
-        <v>26051154M47D2S</v>
+        <v/>
       </c>
       <c r="I2101" t="str">
         <v>pix</v>
@@ -89876,7 +89876,7 @@
         <v>8.43</v>
       </c>
       <c r="H2102" t="str">
-        <v>26051023Y32UH6</v>
+        <v/>
       </c>
       <c r="I2102" t="str">
         <v>pix</v>
@@ -91181,7 +91181,7 @@
         <v>295.51</v>
       </c>
       <c r="H2147" t="str">
-        <v>260520TGBK12TA</v>
+        <v/>
       </c>
       <c r="I2147" t="str">
         <v>pix</v>
@@ -91210,7 +91210,7 @@
         <v>295.51</v>
       </c>
       <c r="H2148" t="str">
-        <v>260520TGBK12TB</v>
+        <v/>
       </c>
       <c r="I2148" t="str">
         <v>pix</v>
@@ -91239,7 +91239,7 @@
         <v>7.94</v>
       </c>
       <c r="H2149" t="str">
-        <v>260515EU5QUHSW</v>
+        <v/>
       </c>
       <c r="I2149" t="str">
         <v>pix</v>
@@ -91268,7 +91268,7 @@
         <v>7.18</v>
       </c>
       <c r="H2150" t="str">
-        <v>260526DTGJEGPQ</v>
+        <v/>
       </c>
       <c r="I2150" t="str">
         <v>pix</v>
@@ -91297,7 +91297,7 @@
         <v>23.75</v>
       </c>
       <c r="H2151" t="str">
-        <v>260528HKCF4DH2</v>
+        <v/>
       </c>
       <c r="I2151" t="str">
         <v>pix</v>
@@ -91326,7 +91326,7 @@
         <v>44.71</v>
       </c>
       <c r="H2152" t="str">
-        <v>260531S85XH2CM</v>
+        <v/>
       </c>
       <c r="I2152" t="str">
         <v>pix</v>
@@ -91355,7 +91355,7 @@
         <v>23.75</v>
       </c>
       <c r="H2153" t="str">
-        <v>260531U9XWGJNQ</v>
+        <v/>
       </c>
       <c r="I2153" t="str">
         <v>money</v>
@@ -91384,7 +91384,7 @@
         <v>23.75</v>
       </c>
       <c r="H2154" t="str">
-        <v>260525C758V5PB</v>
+        <v/>
       </c>
       <c r="I2154" t="str">
         <v>money</v>
@@ -91413,7 +91413,7 @@
         <v>7.18</v>
       </c>
       <c r="H2155" t="str">
-        <v>260527FM7VYVW5</v>
+        <v/>
       </c>
       <c r="I2155" t="str">
         <v>money</v>
@@ -91442,7 +91442,7 @@
         <v>23.75</v>
       </c>
       <c r="H2156" t="str">
-        <v>260531UBQR4QEB</v>
+        <v/>
       </c>
       <c r="I2156" t="str">
         <v>money</v>
@@ -91471,7 +91471,7 @@
         <v>23.75</v>
       </c>
       <c r="H2157" t="str">
-        <v>260529MV79AB08</v>
+        <v/>
       </c>
       <c r="I2157" t="str">
         <v>money</v>
@@ -91500,7 +91500,7 @@
         <v>37.25</v>
       </c>
       <c r="H2158" t="str">
-        <v>260526D8R6YTW1</v>
+        <v/>
       </c>
       <c r="I2158" t="str">
         <v>money</v>
@@ -91529,7 +91529,7 @@
         <v>23.75</v>
       </c>
       <c r="H2159" t="str">
-        <v>2605248BHY5FNX</v>
+        <v/>
       </c>
       <c r="I2159" t="str">
         <v>money</v>
@@ -91558,7 +91558,7 @@
         <v>23.75</v>
       </c>
       <c r="H2160" t="str">
-        <v>260529PCMCB6M5</v>
+        <v/>
       </c>
       <c r="I2160" t="str">
         <v>money</v>
@@ -91587,7 +91587,7 @@
         <v>7.67</v>
       </c>
       <c r="H2161" t="str">
-        <v>260528J1MSR1WM</v>
+        <v/>
       </c>
       <c r="I2161" t="str">
         <v>money</v>
@@ -91616,7 +91616,7 @@
         <v>23.75</v>
       </c>
       <c r="H2162" t="str">
-        <v>260529MJP3NUNV</v>
+        <v/>
       </c>
       <c r="I2162" t="str">
         <v>money</v>
@@ -91645,7 +91645,7 @@
         <v>7.67</v>
       </c>
       <c r="H2163" t="str">
-        <v>260529P78M9G45</v>
+        <v/>
       </c>
       <c r="I2163" t="str">
         <v>money</v>
@@ -91674,7 +91674,7 @@
         <v>23.75</v>
       </c>
       <c r="H2164" t="str">
-        <v>260529NXFECXMX</v>
+        <v/>
       </c>
       <c r="I2164" t="str">
         <v>money</v>
@@ -91703,7 +91703,7 @@
         <v>23.75</v>
       </c>
       <c r="H2165" t="str">
-        <v>260601UG0U18WR</v>
+        <v/>
       </c>
       <c r="I2165" t="str">
         <v>money</v>
@@ -91732,7 +91732,7 @@
         <v>23.75</v>
       </c>
       <c r="H2166" t="str">
-        <v>260601UGBQ39NJ</v>
+        <v/>
       </c>
       <c r="I2166" t="str">
         <v>money</v>
@@ -91761,7 +91761,7 @@
         <v>23.75</v>
       </c>
       <c r="H2167" t="str">
-        <v>260601UKQAUR2H</v>
+        <v/>
       </c>
       <c r="I2167" t="str">
         <v>money</v>
@@ -91790,7 +91790,7 @@
         <v>44.71</v>
       </c>
       <c r="H2168" t="str">
-        <v>260601UXGQ01BJ</v>
+        <v/>
       </c>
       <c r="I2168" t="str">
         <v>money</v>
@@ -91819,7 +91819,7 @@
         <v>7.67</v>
       </c>
       <c r="H2169" t="str">
-        <v>2606010MJDNVMR</v>
+        <v/>
       </c>
       <c r="I2169" t="str">
         <v>money</v>
@@ -91848,7 +91848,7 @@
         <v>7.67</v>
       </c>
       <c r="H2170" t="str">
-        <v>260529MB8B6BM6</v>
+        <v/>
       </c>
       <c r="I2170" t="str">
         <v>money</v>
@@ -91877,7 +91877,7 @@
         <v>23.75</v>
       </c>
       <c r="H2171" t="str">
-        <v>260530PMRMR99A</v>
+        <v/>
       </c>
       <c r="I2171" t="str">
         <v>money</v>
@@ -91906,7 +91906,7 @@
         <v>23.75</v>
       </c>
       <c r="H2172" t="str">
-        <v>260602355XYHPS</v>
+        <v/>
       </c>
       <c r="I2172" t="str">
         <v>money</v>
@@ -91935,7 +91935,7 @@
         <v>23.75</v>
       </c>
       <c r="H2173" t="str">
-        <v>2606021D7H2QCC</v>
+        <v/>
       </c>
       <c r="I2173" t="str">
         <v>money</v>
@@ -91964,7 +91964,7 @@
         <v>7.67</v>
       </c>
       <c r="H2174" t="str">
-        <v>2606020YFPP4MQ</v>
+        <v/>
       </c>
       <c r="I2174" t="str">
         <v>money</v>
@@ -91993,7 +91993,7 @@
         <v>7.67</v>
       </c>
       <c r="H2175" t="str">
-        <v>2606034202M90X</v>
+        <v/>
       </c>
       <c r="I2175" t="str">
         <v>money</v>
@@ -92022,7 +92022,7 @@
         <v>285.6</v>
       </c>
       <c r="H2176" t="str">
-        <v>2606035MGQMDYY</v>
+        <v/>
       </c>
       <c r="I2176" t="str">
         <v>money</v>
@@ -92051,7 +92051,7 @@
         <v>135.6</v>
       </c>
       <c r="H2177" t="str">
-        <v>2606045XY8MGF4</v>
+        <v/>
       </c>
       <c r="I2177" t="str">
         <v>money</v>
@@ -92080,7 +92080,7 @@
         <v>101.6</v>
       </c>
       <c r="H2178" t="str">
-        <v>2606045Y090WHW</v>
+        <v/>
       </c>
       <c r="I2178" t="str">
         <v>money</v>
@@ -92109,7 +92109,7 @@
         <v>23.75</v>
       </c>
       <c r="H2179" t="str">
-        <v>2606033UE8PV0V</v>
+        <v/>
       </c>
       <c r="I2179" t="str">
         <v>money</v>
@@ -92138,7 +92138,7 @@
         <v>23.75</v>
       </c>
       <c r="H2180" t="str">
-        <v>2606035KKVFRNU</v>
+        <v/>
       </c>
       <c r="I2180" t="str">
         <v>money</v>
@@ -92167,7 +92167,7 @@
         <v>23.75</v>
       </c>
       <c r="H2181" t="str">
-        <v>2606046MGAH404</v>
+        <v/>
       </c>
       <c r="I2181" t="str">
         <v>money</v>
@@ -92196,7 +92196,7 @@
         <v>23.75</v>
       </c>
       <c r="H2182" t="str">
-        <v>260606B1XKPJYT</v>
+        <v/>
       </c>
       <c r="I2182" t="str">
         <v>money</v>
@@ -92225,7 +92225,7 @@
         <v>23.75</v>
       </c>
       <c r="H2183" t="str">
-        <v>260606B6MYY3DX</v>
+        <v/>
       </c>
       <c r="I2183" t="str">
         <v>money</v>
@@ -92254,7 +92254,7 @@
         <v>23.75</v>
       </c>
       <c r="H2184" t="str">
-        <v>2606046P31KQAH</v>
+        <v/>
       </c>
       <c r="I2184" t="str">
         <v>money</v>
@@ -92283,7 +92283,7 @@
         <v>23.75</v>
       </c>
       <c r="H2185" t="str">
-        <v>2606058PUG6HXN</v>
+        <v/>
       </c>
       <c r="I2185" t="str">
         <v>money</v>
@@ -92312,7 +92312,7 @@
         <v>23.75</v>
       </c>
       <c r="H2186" t="str">
-        <v>260606B1FWFNXG</v>
+        <v/>
       </c>
       <c r="I2186" t="str">
         <v>money</v>
@@ -92341,7 +92341,7 @@
         <v>7.67</v>
       </c>
       <c r="H2187" t="str">
-        <v>26060590G5B9P4</v>
+        <v/>
       </c>
       <c r="I2187" t="str">
         <v>money</v>
@@ -92370,7 +92370,7 @@
         <v>4</v>
       </c>
       <c r="H2188" t="str">
-        <v>260606AY2SD1DW</v>
+        <v/>
       </c>
       <c r="I2188" t="str">
         <v>money</v>
@@ -92399,7 +92399,7 @@
         <v>3.5</v>
       </c>
       <c r="H2189" t="str">
-        <v>26060481Y18VMK</v>
+        <v/>
       </c>
       <c r="I2189" t="str">
         <v>money</v>
@@ -92428,7 +92428,7 @@
         <v>45.2</v>
       </c>
       <c r="H2190" t="str">
-        <v>260606BPCWMEVU</v>
+        <v/>
       </c>
       <c r="I2190" t="str">
         <v>money</v>

</xml_diff>